<commit_message>
Add test report, test script & automation video for TS01
</commit_message>
<xml_diff>
--- a/Test-cases/Test Scenario 01 - Search functionality.xlsx
+++ b/Test-cases/Test Scenario 01 - Search functionality.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ThemoviedbTesting\Test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B0C44C8-9B5B-4A47-B609-64A0725F3334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AC05DE0-C917-4853-A993-2A873713F6F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3450" yWindow="3525" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Case Template" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="106">
   <si>
     <t>Test Scenario ID</t>
   </si>
@@ -270,9 +270,6 @@
 2. Press Enter</t>
   </si>
   <si>
-    <t>"映画"</t>
-  </si>
-  <si>
     <t xml:space="preserve">No results found' message displayed
 </t>
   </si>
@@ -292,9 +289,6 @@
 2. Press Enter</t>
   </si>
   <si>
-    <t>"    Avengers     "</t>
-  </si>
-  <si>
     <t xml:space="preserve">Results same as searching 'Avengers' — spaces trimmed
 </t>
   </si>
@@ -310,9 +304,6 @@
 2. Press Enter</t>
   </si>
   <si>
-    <t>"a"</t>
-  </si>
-  <si>
     <t xml:space="preserve">Results page loads with movies containing 'a'; pagination available
 </t>
   </si>
@@ -328,9 +319,6 @@
 2. Press Enter</t>
   </si>
   <si>
-    <t>"2024"</t>
-  </si>
-  <si>
     <t xml:space="preserve">Results include movies with '2024' in title
 </t>
   </si>
@@ -346,9 +334,6 @@
 2. Press Enter</t>
   </si>
   <si>
-    <t>"Breaking Bad"</t>
-  </si>
-  <si>
     <t xml:space="preserve">TV Shows tab shows relevant TV show results
 </t>
   </si>
@@ -362,9 +347,6 @@
   <si>
     <t>1. Search 'Tom Hanks'
 2. Press Enter</t>
-  </si>
-  <si>
-    <t>"Tom Hanks"</t>
   </si>
   <si>
     <t xml:space="preserve">People tab shows Tom Hanks and related people
@@ -393,6 +375,21 @@
   </si>
   <si>
     <t>Vu Dinh Duy</t>
+  </si>
+  <si>
+    <t>映画</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>Tom Hanks</t>
+  </si>
+  <si>
+    <t>Breaking Bad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Avengers     </t>
   </si>
 </sst>
 </file>
@@ -603,7 +600,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -649,13 +646,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -663,12 +657,14 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -678,8 +674,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -918,10 +918,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
+      <c r="B1" s="27"/>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
@@ -929,14 +929,14 @@
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:17">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="28"/>
+      <c r="B2" s="27"/>
       <c r="C2" s="3" t="s">
         <v>4</v>
       </c>
@@ -948,10 +948,10 @@
       </c>
     </row>
     <row r="3" spans="1:17">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="28"/>
+      <c r="B3" s="27"/>
       <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
@@ -967,18 +967,18 @@
       <c r="D4" s="5"/>
     </row>
     <row r="5" spans="1:17" ht="15" customHeight="1">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="31"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
+      <c r="J5" s="30"/>
     </row>
     <row r="6" spans="1:17">
       <c r="A6" s="6" t="s">
@@ -1011,8 +1011,8 @@
       <c r="J6" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="M6" s="25"/>
-      <c r="N6" s="26"/>
+      <c r="M6" s="31"/>
+      <c r="N6" s="32"/>
       <c r="O6" s="5"/>
       <c r="P6" s="7"/>
       <c r="Q6" s="5"/>
@@ -1044,8 +1044,8 @@
       </c>
       <c r="I7" s="8"/>
       <c r="J7" s="8"/>
-      <c r="M7" s="25"/>
-      <c r="N7" s="26"/>
+      <c r="M7" s="31"/>
+      <c r="N7" s="32"/>
       <c r="O7" s="5"/>
       <c r="P7" s="7"/>
       <c r="Q7" s="13"/>
@@ -1191,32 +1191,32 @@
       <c r="J12" s="15"/>
     </row>
     <row r="13" spans="1:17" ht="30" customHeight="1">
-      <c r="A13" s="23" t="s">
+      <c r="A13" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="B13" s="23" t="s">
+      <c r="B13" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="22" t="s">
         <v>60</v>
       </c>
       <c r="D13" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="E13" s="23" t="s">
+      <c r="E13" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="F13" s="23" t="s">
+      <c r="F13" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="H13" s="21" t="s">
+      <c r="H13" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="I13" s="22"/>
-      <c r="J13" s="22"/>
+      <c r="I13" s="21"/>
+      <c r="J13" s="21"/>
     </row>
     <row r="14" spans="1:17">
       <c r="A14" s="20"/>
@@ -1231,32 +1231,32 @@
       <c r="J14" s="20"/>
     </row>
     <row r="15" spans="1:17" ht="15" customHeight="1">
-      <c r="A15" s="23" t="s">
+      <c r="A15" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="B15" s="23" t="s">
+      <c r="B15" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="C15" s="23" t="s">
+      <c r="C15" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="D15" s="23" t="s">
+      <c r="D15" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="E15" s="23" t="s">
+      <c r="E15" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="F15" s="23" t="s">
+      <c r="F15" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="G15" s="19" t="s">
+      <c r="G15" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="H15" s="21" t="s">
+      <c r="H15" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="I15" s="22"/>
-      <c r="J15" s="22"/>
+      <c r="I15" s="21"/>
+      <c r="J15" s="21"/>
     </row>
     <row r="16" spans="1:17">
       <c r="A16" s="20"/>
@@ -1271,32 +1271,32 @@
       <c r="J16" s="20"/>
     </row>
     <row r="17" spans="1:10" ht="15" customHeight="1">
-      <c r="A17" s="23" t="s">
+      <c r="A17" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="B17" s="23" t="s">
+      <c r="B17" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="C17" s="22" t="s">
         <v>60</v>
       </c>
       <c r="D17" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="E17" s="23" t="s">
+      <c r="E17" s="22" t="s">
+        <v>101</v>
+      </c>
+      <c r="F17" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="F17" s="32" t="s">
+      <c r="G17" s="23" t="s">
         <v>74</v>
       </c>
-      <c r="G17" s="19" t="s">
-        <v>75</v>
-      </c>
-      <c r="H17" s="21" t="s">
+      <c r="H17" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="I17" s="22"/>
-      <c r="J17" s="22"/>
+      <c r="I17" s="21"/>
+      <c r="J17" s="21"/>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="20"/>
@@ -1312,22 +1312,22 @@
     </row>
     <row r="19" spans="1:10" ht="30">
       <c r="A19" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" s="9" t="s">
         <v>76</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>77</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>60</v>
       </c>
       <c r="D19" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="F19" s="9" t="s">
         <v>78</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="F19" s="9" t="s">
-        <v>80</v>
       </c>
       <c r="G19" s="18" t="s">
         <v>27</v>
@@ -1340,22 +1340,22 @@
     </row>
     <row r="20" spans="1:10" ht="30">
       <c r="A20" s="9" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>60</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G20" s="18" t="s">
         <v>27</v>
@@ -1368,22 +1368,22 @@
     </row>
     <row r="21" spans="1:10" ht="15.75" customHeight="1">
       <c r="A21" s="16" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C21" s="16" t="s">
         <v>60</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="E21" s="16" t="s">
-        <v>89</v>
+        <v>85</v>
+      </c>
+      <c r="E21" s="33">
+        <v>2024</v>
       </c>
       <c r="F21" s="16" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="G21" s="18" t="s">
         <v>27</v>
@@ -1395,32 +1395,32 @@
       <c r="J21" s="15"/>
     </row>
     <row r="22" spans="1:10" ht="15.75" customHeight="1">
-      <c r="A22" s="23" t="s">
-        <v>91</v>
-      </c>
-      <c r="B22" s="23" t="s">
-        <v>92</v>
-      </c>
-      <c r="C22" s="23" t="s">
+      <c r="A22" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="B22" s="22" t="s">
+        <v>88</v>
+      </c>
+      <c r="C22" s="22" t="s">
         <v>60</v>
       </c>
       <c r="D22" s="24" t="s">
-        <v>93</v>
-      </c>
-      <c r="E22" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="F22" s="23" t="s">
-        <v>95</v>
-      </c>
-      <c r="G22" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="E22" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="F22" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="G22" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="H22" s="21" t="s">
+      <c r="H22" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="I22" s="22"/>
-      <c r="J22" s="22"/>
+      <c r="I22" s="21"/>
+      <c r="J22" s="21"/>
     </row>
     <row r="23" spans="1:10" ht="15.75" customHeight="1">
       <c r="A23" s="20"/>
@@ -1435,32 +1435,32 @@
       <c r="J23" s="20"/>
     </row>
     <row r="24" spans="1:10" ht="15.75" customHeight="1">
-      <c r="A24" s="23" t="s">
-        <v>96</v>
-      </c>
-      <c r="B24" s="23" t="s">
-        <v>97</v>
-      </c>
-      <c r="C24" s="23" t="s">
+      <c r="A24" s="22" t="s">
+        <v>91</v>
+      </c>
+      <c r="B24" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="C24" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="D24" s="23" t="s">
-        <v>98</v>
-      </c>
-      <c r="E24" s="23" t="s">
-        <v>99</v>
-      </c>
-      <c r="F24" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="G24" s="19" t="s">
+      <c r="D24" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="E24" s="22" t="s">
+        <v>103</v>
+      </c>
+      <c r="F24" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="G24" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="H24" s="21" t="s">
+      <c r="H24" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="I24" s="22"/>
-      <c r="J24" s="22"/>
+      <c r="I24" s="21"/>
+      <c r="J24" s="21"/>
     </row>
     <row r="25" spans="1:10" ht="15.75" customHeight="1">
       <c r="A25" s="20"/>
@@ -1475,32 +1475,32 @@
       <c r="J25" s="20"/>
     </row>
     <row r="26" spans="1:10" ht="15.75" customHeight="1">
-      <c r="A26" s="23" t="s">
-        <v>101</v>
-      </c>
-      <c r="B26" s="23" t="s">
+      <c r="A26" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="B26" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="C26" s="22" t="s">
+        <v>97</v>
+      </c>
+      <c r="D26" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="E26" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="C26" s="23" t="s">
-        <v>103</v>
-      </c>
-      <c r="D26" s="24" t="s">
-        <v>104</v>
-      </c>
-      <c r="E26" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="F26" s="23" t="s">
-        <v>105</v>
-      </c>
-      <c r="G26" s="19" t="s">
+      <c r="F26" s="22" t="s">
+        <v>99</v>
+      </c>
+      <c r="G26" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="H26" s="21" t="s">
+      <c r="H26" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="I26" s="22"/>
-      <c r="J26" s="22"/>
+      <c r="I26" s="21"/>
+      <c r="J26" s="21"/>
     </row>
     <row r="27" spans="1:10" ht="43.5" customHeight="1">
       <c r="A27" s="20"/>
@@ -5408,34 +5408,28 @@
     </row>
   </sheetData>
   <mergeCells count="66">
-    <mergeCell ref="H24:H25"/>
-    <mergeCell ref="I24:I25"/>
-    <mergeCell ref="J24:J25"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="F24:F25"/>
-    <mergeCell ref="G24:G25"/>
-    <mergeCell ref="H26:H27"/>
-    <mergeCell ref="I26:I27"/>
-    <mergeCell ref="J26:J27"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="E26:E27"/>
-    <mergeCell ref="F26:F27"/>
-    <mergeCell ref="G26:G27"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="H22:H23"/>
+    <mergeCell ref="I22:I23"/>
+    <mergeCell ref="J22:J23"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="F22:F23"/>
+    <mergeCell ref="H17:H18"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
@@ -5452,28 +5446,34 @@
     <mergeCell ref="G13:G14"/>
     <mergeCell ref="F15:F16"/>
     <mergeCell ref="G15:G16"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="G22:G23"/>
-    <mergeCell ref="H22:H23"/>
-    <mergeCell ref="I22:I23"/>
-    <mergeCell ref="J22:J23"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A22:A23"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="E22:E23"/>
-    <mergeCell ref="F22:F23"/>
-    <mergeCell ref="H17:H18"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="H26:H27"/>
+    <mergeCell ref="I26:I27"/>
+    <mergeCell ref="J26:J27"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="E26:E27"/>
+    <mergeCell ref="F26:F27"/>
+    <mergeCell ref="G26:G27"/>
+    <mergeCell ref="H24:H25"/>
+    <mergeCell ref="I24:I25"/>
+    <mergeCell ref="J24:J25"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="F24:F25"/>
+    <mergeCell ref="G24:G25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>